<commit_message>
Data and Analysis for Each Sensor
Data and Analysis for Each Sensor
</commit_message>
<xml_diff>
--- a/Data for Sensors Project GitHub.xlsx
+++ b/Data for Sensors Project GitHub.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/393eb17cc9944417/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\iamam\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{FF4562E3-244D-487F-B9A7-644D43BA3BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A3DA69E-5653-4985-B769-7362BA1EE0A7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A92698DB-5C41-4424-A804-22A874F1DB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-3160" yWindow="10690" windowWidth="25820" windowHeight="13900" tabRatio="594" xr2:uid="{4F754F05-7713-4394-AA0D-BE8A2C49AABA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="594" activeTab="2" xr2:uid="{4F754F05-7713-4394-AA0D-BE8A2C49AABA}"/>
   </bookViews>
   <sheets>
     <sheet name="MPU Accuracy" sheetId="12" r:id="rId1"/>
@@ -13784,34 +13784,34 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
                 <c:pt idx="0">
-                  <c:v>4.1066666666666674</c:v>
+                  <c:v>43.906666666666666</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>9.3533333333333353</c:v>
+                  <c:v>45.796666666666667</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.2966666666666642</c:v>
+                  <c:v>45.928333333333335</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.416666666666667</c:v>
+                  <c:v>49.891666666666666</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8.4333333333333353</c:v>
+                  <c:v>54.846666666666664</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>11.019999999999998</c:v>
+                  <c:v>57.81</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>9.0250000000000004</c:v>
+                  <c:v>56.841666666666669</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>12.200000000000001</c:v>
+                  <c:v>60.8</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>11.573333333333336</c:v>
+                  <c:v>61.813333333333333</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>28.746666666666663</c:v>
+                  <c:v>76.626666666666665</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -19505,12 +19505,11 @@
         <v>1.7372000000000001</v>
       </c>
       <c r="AK2">
-        <f>4*9.81</f>
-        <v>39.24</v>
+        <v>4</v>
       </c>
       <c r="AL2" s="16">
         <f>AJ2/AK2</f>
-        <v>4.4271151885830785E-2</v>
+        <v>0.43430000000000002</v>
       </c>
     </row>
     <row r="3" spans="1:38" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
@@ -49384,8 +49383,8 @@
         <v>0.64400000000000002</v>
       </c>
       <c r="Q19">
-        <f t="shared" si="3"/>
-        <v>4.1066666666666674</v>
+        <f>ABS(K19-D19)</f>
+        <v>43.906666666666666</v>
       </c>
       <c r="S19">
         <f>AVERAGE(P19:P28)</f>
@@ -49393,7 +49392,7 @@
       </c>
       <c r="T19">
         <f>AVERAGE(Q19:Q31)</f>
-        <v>10.317166666666665</v>
+        <v>55.426166666666667</v>
       </c>
     </row>
     <row r="20" spans="2:20" x14ac:dyDescent="0.2">
@@ -49431,8 +49430,8 @@
         <v>1.036</v>
       </c>
       <c r="Q20">
-        <f t="shared" si="3"/>
-        <v>9.3533333333333353</v>
+        <f>ABS(K20-D20)</f>
+        <v>45.796666666666667</v>
       </c>
     </row>
     <row r="21" spans="2:20" x14ac:dyDescent="0.2">
@@ -49470,8 +49469,8 @@
         <v>0.33600000000000008</v>
       </c>
       <c r="Q21">
-        <f t="shared" si="3"/>
-        <v>3.2966666666666642</v>
+        <f t="shared" ref="Q21:Q28" si="6">ABS(K21-D21)</f>
+        <v>45.928333333333335</v>
       </c>
     </row>
     <row r="22" spans="2:20" x14ac:dyDescent="0.2">
@@ -49509,8 +49508,8 @@
         <v>0.3239999999999999</v>
       </c>
       <c r="Q22">
-        <f t="shared" si="3"/>
-        <v>5.416666666666667</v>
+        <f t="shared" si="6"/>
+        <v>49.891666666666666</v>
       </c>
     </row>
     <row r="23" spans="2:20" x14ac:dyDescent="0.2">
@@ -49548,8 +49547,8 @@
         <v>0.25</v>
       </c>
       <c r="Q23">
-        <f t="shared" si="3"/>
-        <v>8.4333333333333353</v>
+        <f t="shared" si="6"/>
+        <v>54.846666666666664</v>
       </c>
     </row>
     <row r="24" spans="2:20" x14ac:dyDescent="0.2">
@@ -49587,8 +49586,8 @@
         <v>0.26400000000000001</v>
       </c>
       <c r="Q24">
-        <f t="shared" si="3"/>
-        <v>11.019999999999998</v>
+        <f t="shared" si="6"/>
+        <v>57.81</v>
       </c>
     </row>
     <row r="25" spans="2:20" x14ac:dyDescent="0.2">
@@ -49626,8 +49625,8 @@
         <v>0.26400000000000001</v>
       </c>
       <c r="Q25">
-        <f t="shared" si="3"/>
-        <v>9.0250000000000004</v>
+        <f t="shared" si="6"/>
+        <v>56.841666666666669</v>
       </c>
     </row>
     <row r="26" spans="2:20" x14ac:dyDescent="0.2">
@@ -49665,8 +49664,8 @@
         <v>0.19200000000000003</v>
       </c>
       <c r="Q26">
-        <f t="shared" si="3"/>
-        <v>12.200000000000001</v>
+        <f t="shared" si="6"/>
+        <v>60.8</v>
       </c>
     </row>
     <row r="27" spans="2:20" x14ac:dyDescent="0.2">
@@ -49704,8 +49703,8 @@
         <v>0.16799999999999998</v>
       </c>
       <c r="Q27">
-        <f t="shared" si="3"/>
-        <v>11.573333333333336</v>
+        <f t="shared" si="6"/>
+        <v>61.813333333333333</v>
       </c>
     </row>
     <row r="28" spans="2:20" x14ac:dyDescent="0.2">
@@ -49743,8 +49742,8 @@
         <v>0.15599999999999997</v>
       </c>
       <c r="Q28">
-        <f t="shared" si="3"/>
-        <v>28.746666666666663</v>
+        <f t="shared" si="6"/>
+        <v>76.626666666666665</v>
       </c>
     </row>
   </sheetData>
@@ -50034,6 +50033,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="7552e3d3-701d-4b50-a6fe-9ca124d198dd" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010046215E641A850F40840E9D6E0F2AA5A4" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="db4aa90056b5712bf55e6ff347ff4a5a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="7552e3d3-701d-4b50-a6fe-9ca124d198dd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="83165ff45b7db376f9566712734db917" ns3:_="">
     <xsd:import namespace="7552e3d3-701d-4b50-a6fe-9ca124d198dd"/>
@@ -50215,7 +50222,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -50224,15 +50231,23 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="7552e3d3-701d-4b50-a6fe-9ca124d198dd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{359801A8-9908-4405-BE6A-C356DDACA95D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="7552e3d3-701d-4b50-a6fe-9ca124d198dd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{18343AD3-3FCE-4AE0-A089-106C63D347D0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -50250,26 +50265,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DAEF504B-F3F9-471C-9A55-A3A0B72A4E39}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{359801A8-9908-4405-BE6A-C356DDACA95D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="7552e3d3-701d-4b50-a6fe-9ca124d198dd"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>